<commit_message>
Adding the updated  report part
</commit_message>
<xml_diff>
--- a/test_data/data_quality_requirements.xlsx
+++ b/test_data/data_quality_requirements.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180"/>
+    <workbookView windowWidth="27945" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="DQ_REQUIREMENTS" sheetId="1" r:id="rId1"/>
     <sheet name="INSTRUCTIONS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DQ_REQUIREMENTS!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DQ_REQUIREMENTS!$A$1:$I$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="30">
   <si>
     <t>SlNO</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>PHONE</t>
+  </si>
+  <si>
+    <t>CUSTOMER_ID</t>
   </si>
   <si>
     <t>Column</t>
@@ -1097,8 +1100,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="22" customWidth="1"/>
@@ -1225,8 +1228,37 @@
         <v>11</v>
       </c>
     </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I4" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I5" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <dataValidations count="3">
@@ -1257,10 +1289,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1268,23 +1300,23 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1292,7 +1324,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1300,7 +1332,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1308,7 +1340,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1316,7 +1348,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1324,7 +1356,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1332,7 +1364,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>